<commit_message>
Daily check, Verified tick, download names and links
- The weekly check is now the daily check (engine/weekly.py renamed
  engine/daily.py), run every day at 11:15 am; its sample changes daily.
- After a check passes, the app shows a green Verified tick with the
  time of that check, until the next check.
- Downloads are named brand_day-of-fetch (e.g. Bhama_30-09-2026.xlsx);
  every price in the Excel file links to the page it was read from.
- The spot-check's page script skips hidden elements (Bhama's hidden
  struck copy of the sale price was read as the MRP).
- Brand catalogue: Bhama added.
</commit_message>
<xml_diff>
--- a/data/brand_catalogue.xlsx
+++ b/data/brand_catalogue.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vastramay" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BownBee" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AJ Dezines" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bhama" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7781,7 +7782,6 @@
           <t>Pink Cotton 3/4th Sleeves Floral Printed Girls Suit Set with Sequins Lace Work</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122670/zoddle/img-5640f489.jpg</t>
@@ -7797,7 +7797,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-pink-floral-printed-cotton-kurta-with-sharara--dupatta-set/37245250/buy</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0G5ZCNZ4S</t>
@@ -7841,7 +7840,6 @@
           <t>Pink Cotton 3/4th Sleeves Floral Printed Girls Suit Set with Sequins Lace Work</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122670/zoddle/img-5640f489.jpg</t>
@@ -7857,7 +7855,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-pink-floral-printed-cotton-kurta-with-sharara--dupatta-set/37245250/buy</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0G5ZCNZ4S</t>
@@ -7901,7 +7898,6 @@
           <t>Girls Green Cotton Three-Fourth Sleeves Floral Printed Girls Suit Set</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122667/zoddle/img-65ddd03b.jpg</t>
@@ -7917,8 +7913,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-paisley-printed-empire-a-line-pure-cotton-kurta-with-palazzos--dupatta-set/37190084/buy</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-sharara-set/p/itm5bb45dc3d73f8</t>
@@ -7957,7 +7951,6 @@
           <t>Dark Green Cotton Sleeveless Lurex and Gotta Work Girls Suit Set</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122666/zoddle/img-fed2d072.jpg</t>
@@ -7973,8 +7966,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-green-striped-gotta-patti-pure-cotton-anarkali-kurta-with-palazzos-set/36360308/buy</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-sharara-set/p/itm936a4df991784</t>
@@ -8013,7 +8004,6 @@
           <t>Dark Green Cotton Sleeveless Lurex and Gotta Work Girls Suit Set</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122666/zoddle/img-fed2d072.jpg</t>
@@ -8029,8 +8019,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-green-striped-gotta-patti-pure-cotton-anarkali-kurta-with-palazzos-set/36360308/buy</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-sharara-set/p/itm936a4df991784</t>
@@ -8069,7 +8057,6 @@
           <t>Maroon Cotton Sleeveless Lurex and Gotta Work Girls Suit Set</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122646/zoddle/img-84c7c02c.jpg</t>
@@ -8085,8 +8072,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-striped-gotta-patti-pure-cotton-anarkali-kurta-with-sharara--dupatta-set/36360300/buy</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-sharara-set/p/itm48699df767266</t>
@@ -8125,7 +8110,6 @@
           <t>Maroon Cotton Sleeveless Lurex and Gotta Work Girls Suit Set</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122646/zoddle/img-84c7c02c.jpg</t>
@@ -8141,8 +8125,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-striped-gotta-patti-pure-cotton-anarkali-kurta-with-sharara--dupatta-set/36360300/buy</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-sharara-set/p/itm48699df767266</t>
@@ -8181,7 +8163,6 @@
           <t>Girls Firozi Foil Print Georgette Sharara for Kids</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122663/zoddle/img-8f2120fd.jpg</t>
@@ -8245,7 +8226,6 @@
           <t>Girls Firozi Foil Print Georgette Sharara for Kids</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122663/zoddle/img-8f2120fd.jpg</t>
@@ -8309,7 +8289,6 @@
           <t>Maroon Velvet Full Sleeves Solid Girls Suit Set</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122652/zoddle/img-3d152af9.jpg</t>
@@ -8325,7 +8304,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-regular-gotta-patti-velvet-kurta-with-trousers/39203153/buy</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GHS4RJT4</t>
@@ -8369,7 +8347,6 @@
           <t>Maroon Velvet Full Sleeves Solid Girls Suit Set</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122652/zoddle/img-3d152af9.jpg</t>
@@ -8385,7 +8362,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-regular-gotta-patti-velvet-kurta-with-trousers/39203153/buy</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GHS4RJT4</t>
@@ -8429,7 +8405,6 @@
           <t>Maroon Velvet Full Sleeves Solid Girls Suit Set</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122652/zoddle/img-3d152af9.jpg</t>
@@ -8445,7 +8420,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-regular-gotta-patti-velvet-kurta-with-trousers/39203153/buy</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GHS4RJT4</t>
@@ -8489,7 +8463,6 @@
           <t>Pink Polka Dots and Floral Print Silk blend Kurti Palazzo and Dupatta For Girls</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122671/zoddle/img-c52b709e.jpg</t>
@@ -8505,8 +8478,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-ethnic-motifs-printed-regular-kurta-with-palazzos--with-dupatta/45627846/buy</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-palazzo-set/p/itmc77c9c4543329</t>
@@ -8545,7 +8516,6 @@
           <t>Red Heavy Embroidered Brocade Kurti and Palazzo For Girls</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122672/zoddle/img-1286a45e.jpg</t>
@@ -8561,8 +8531,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-floral-regular-kurti-with-palazzos/40493952/buy</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-palazzo-set/p/itm0f349dd9b20b6</t>
@@ -8601,20 +8569,16 @@
           <t>Pink Lurex Work Cotton Girls Suit Set For Girls</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122673/zoddle/img-2c4b3703.jpg</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-girls-striped-tiered-pure-cotton-kurti-with-sharara--with-dupatta/40869762/buy</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-girls-festive-party-kurta-sharara-set/p/itm490c5eb4d9b64</t>
@@ -8653,7 +8617,6 @@
           <t>Girls Purple Net Sleeveless Heavy Embroidered Lehenga Choli</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122675/zoddle/img-34f78e5b.jpg</t>
@@ -8664,8 +8627,6 @@
           <t>https://ajdezines.com/products/girls-purple-net-sleeveless-heavy-embroidered-lehenga-choli</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0G34LXFPB</t>
@@ -8709,7 +8670,6 @@
           <t>Girls Pink Cotton Half-Sleeves Floral Printed Lehenga Choli</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122674/zoddle/img-1cdfec47.jpg</t>
@@ -8725,7 +8685,6 @@
           <t>https://www.myntra.com/lehenga-choli/aj+dezines/aj-dezines-girls-pink-floral-printed-ready-to-wear-cotton-lehenga--blouse-with-dupatta/36605906/buy</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0FQV638BZ</t>
@@ -8769,7 +8728,6 @@
           <t>Girls Pink Cotton Half-Sleeves Floral Printed Lehenga Choli</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122674/zoddle/img-1cdfec47.jpg</t>
@@ -8785,7 +8743,6 @@
           <t>https://www.myntra.com/lehenga-choli/aj+dezines/aj-dezines-girls-pink-floral-printed-ready-to-wear-cotton-lehenga--blouse-with-dupatta/36605906/buy</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0FQV638BZ</t>
@@ -8829,7 +8786,6 @@
           <t>Yellow Cotton Sleeveless Floral Printed Lehenga Choli for Girls</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122678/zoddle/img-180bdec1.jpg</t>
@@ -8845,7 +8801,6 @@
           <t>https://www.myntra.com/lehenga-choli/aj+dezines/aj-dezines-girls-floral-printed-halter-neck-gotta-patti-cotton-ready-to-wear-lehenga-choli/34955993/buy</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0FFN18HQD</t>
@@ -8889,7 +8844,6 @@
           <t>Kids Boys Yellow Cotton Full Sleeves Floral Print Kurta Pyjama Set</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122639/zoddle/img-0be4c895.jpg</t>
@@ -8905,8 +8859,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-floral-printed-kurta-pyjama-set/36003122/buy</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-boys-festive-party-kurta-pyjama-set/p/itm21e99a16eb256</t>
@@ -8945,7 +8897,6 @@
           <t>Multi Foil Print Silk Blend Kurta and Pyjama (Pink)</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122645/zoddle/img-bfcad5b7.jpg</t>
@@ -8956,8 +8907,6 @@
           <t>https://ajdezines.com/products/1302-pink</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GRMZDGWM</t>
@@ -9001,7 +8950,6 @@
           <t>Multi Foil Print Silk Blend Kurta and Pyjama (Pink)</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122645/zoddle/img-bfcad5b7.jpg</t>
@@ -9012,8 +8960,6 @@
           <t>https://ajdezines.com/products/1302-pink</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GRMZDGWM</t>
@@ -9057,7 +9003,6 @@
           <t>Kids Boys PINK Bandhani Print Cotton Kurta Pyjama Set (1247)</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122636/zoddle/img-3a2d2116.jpg</t>
@@ -9073,7 +9018,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-pink-bandhani-printed-mandarin-collar-pure-cotton-kurta-with-pyjamas-set/25431386/buy</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CNRY6DXK</t>
@@ -9117,7 +9061,6 @@
           <t>Kids Boys PINK Bandhani Print Cotton Kurta Pyjama Set (1247)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122636/zoddle/img-3a2d2116.jpg</t>
@@ -9133,7 +9076,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-pink-bandhani-printed-mandarin-collar-pure-cotton-kurta-with-pyjamas-set/25431386/buy</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CNRY6DXK</t>
@@ -9177,7 +9119,6 @@
           <t>Kids Boys Green Embroidered Schiffli Kurta Pyjama Set (1250)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122637/zoddle/img-782ce9af.jpg</t>
@@ -9193,7 +9134,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-ethnic-motifs-sequinned-chikankari-pure-cotton-kurta-with-salwar-set/23921206/buy</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CWRX4VVL</t>
@@ -9237,7 +9177,6 @@
           <t>Kids Boys Green Embroidered Schiffli Kurta Pyjama Set (1250)</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122637/zoddle/img-782ce9af.jpg</t>
@@ -9253,7 +9192,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-ethnic-motifs-sequinned-chikankari-pure-cotton-kurta-with-salwar-set/23921206/buy</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CWRX4VVL</t>
@@ -9297,20 +9235,16 @@
           <t>Yellow Lurex Work Cotton Kurta Pyjama Waist Coat Set For Boys (569)</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122655/zoddle/img-d2bdfab7.jpg</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-striped-regular-pure-cotton-kurta-with-pyjamas/40869763/buy</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-boys-festive-party-kurta-waistcoat-pyjama-set/p/itm8aa18c9c13bb2</t>
@@ -9349,7 +9283,6 @@
           <t>Kids Ethnic Wear Boys Maroon Silk Blend Dhoti Set (1916)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122647/zoddle/img-170a0f41.jpg</t>
@@ -9365,7 +9298,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-solid-kurta-with-dhoti-pants/21338284/buy</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0DF82BZ35</t>
@@ -9409,7 +9341,6 @@
           <t>Kids Ethnic Wear Boys Maroon Silk Blend Dhoti Set (1916)</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122647/zoddle/img-170a0f41.jpg</t>
@@ -9425,7 +9356,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-solid-kurta-with-dhoti-pants/21338284/buy</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0DF82BZ35</t>
@@ -9469,7 +9399,6 @@
           <t>Kids Ethnic Wear Boys Maroon Silk Blend Dhoti Set (1916)</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122647/zoddle/img-170a0f41.jpg</t>
@@ -9485,7 +9414,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-solid-kurta-with-dhoti-pants/21338284/buy</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0DF82BZ35</t>
@@ -9529,7 +9457,6 @@
           <t>Kids Boys Maroon Solid Raw Silk Dhoti Set (1926)</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122648/zoddle/img-14a155be.jpg</t>
@@ -9593,20 +9520,16 @@
           <t>Purple Cotton Full Sleeves Floral Printed Dhoti Set (1959)</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122651/zoddle/img-63f484cd.jpg</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-purple-band-collar-pure-cotton-kurta-with-dhoti-pant--nehru-jacket-set/37705571/buy</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-boys-wedding-kurta-waistcoat-dhoti-pant-set/p/itm7437f8ea6381d</t>
@@ -9645,20 +9568,16 @@
           <t>Purple Cotton Full Sleeves Floral Printed Dhoti Set (1959)</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122651/zoddle/img-63f484cd.jpg</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-purple-band-collar-pure-cotton-kurta-with-dhoti-pant--nehru-jacket-set/37705571/buy</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-boys-wedding-kurta-waistcoat-dhoti-pant-set/p/itm7437f8ea6381d</t>
@@ -9697,7 +9616,6 @@
           <t>Green Cotton Full Sleeves Floral Print Dhoti Kurta (1950)</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122650/zoddle/img-91c8dced.jpg</t>
@@ -9713,8 +9631,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-chevron-printed-long-sleeves-pure-cotton-kurta-with-dhoti-pants/34028117/buy</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-boys-festive-party-dhoti-kurta-set/p/itm6f4f9e440d8b3</t>
@@ -9753,7 +9669,6 @@
           <t>Kids Boys Floral Print Cotton Dhoti Set with Waistcoat (1929)</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122649/zoddle/img-12103823.jpg</t>
@@ -9764,7 +9679,6 @@
           <t>https://ajdezines.com/products/kids-cotton-printed-red-dhoti-kurta-set-for-boys-with-waistcoat</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>https://www.firstcry.com/aj-dezines/aj-dezines-pure-cotton-woven-full-sleeves-floral-printed-jacket-dhoti-set-red-and-navy/24213917/product-detail</t>
@@ -9813,7 +9727,6 @@
           <t>Kids Boys Floral Print Cotton Dhoti Set with Waistcoat (1929)</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122649/zoddle/img-12103823.jpg</t>
@@ -9824,7 +9737,6 @@
           <t>https://ajdezines.com/products/kids-cotton-printed-red-dhoti-kurta-set-for-boys-with-waistcoat</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>https://www.firstcry.com/aj-dezines/aj-dezines-pure-cotton-woven-full-sleeves-floral-printed-jacket-dhoti-set-red-and-navy/24213917/product-detail</t>
@@ -9873,7 +9785,6 @@
           <t>Kids Boys Floral Print Cotton Dhoti Set with Waistcoat (1929)</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122649/zoddle/img-12103823.jpg</t>
@@ -9884,7 +9795,6 @@
           <t>https://ajdezines.com/products/kids-cotton-printed-red-dhoti-kurta-set-for-boys-with-waistcoat</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>https://www.firstcry.com/aj-dezines/aj-dezines-pure-cotton-woven-full-sleeves-floral-printed-jacket-dhoti-set-red-and-navy/24213917/product-detail</t>
@@ -9933,7 +9843,6 @@
           <t>Boys Mustard Solid Silk Sherwani for Kids</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122680/zoddle/img-337e43f7.jpg</t>
@@ -9944,8 +9853,6 @@
           <t>https://ajdezines.com/products/aj-dezines-boys-sherwani-embroidered-mukaish</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0C3HXRSV4</t>
@@ -9989,7 +9896,6 @@
           <t>Navy-blue Printed Silk Blend Sherwani For Boys</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122659/zoddle/img-1333325c.jpg</t>
@@ -10000,8 +9906,6 @@
           <t>https://ajdezines.com/products/7097-navy-blue-sherwani</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GQ46LP84</t>
@@ -10045,7 +9949,6 @@
           <t>Navy-blue Printed Silk Blend Sherwani For Boys</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122659/zoddle/img-1333325c.jpg</t>
@@ -10056,8 +9959,6 @@
           <t>https://ajdezines.com/products/7097-navy-blue-sherwani</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GQ46LP84</t>
@@ -10101,7 +10002,6 @@
           <t>Kids Boys Rust Printed Silk Blend Sherwani</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122657/zoddle/img-051bef6a.jpg</t>
@@ -10165,17 +10065,11 @@
           <t>Pink Jacquard Full Sleeves Sherwani with Rich Floral Embroidery for boys</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122660/zoddle/img-db393a0d.jpg</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -10209,7 +10103,6 @@
           <t>Boys Blue Jacquard Full Sleeves Rich Embroidery Sherwani</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122658/zoddle/img-e24ce0d7.jpg</t>
@@ -10225,9 +10118,6 @@
           <t>https://www.myntra.com/sherwani/aj+dezines/aj-dezines-boys-blue-jacquard-full-sleeves-rich-embroidered-sherwani-set/37420060/buy</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -10261,17 +10151,11 @@
           <t>Kids Boys Green Embroidered Cotton Polyester Sherwani</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122655/zoddle/img-f90f7e5c.jpg</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -10305,7 +10189,6 @@
           <t>Boys Maroon Embroidered Velvet Sherwani for Kids</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122682/zoddle/img-5e3463e2.jpg</t>
@@ -10316,8 +10199,6 @@
           <t>https://ajdezines.com/products/boys-maroon-velvet-embroidered-sequin-sherwani-set</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CSPGVT69</t>
@@ -10361,7 +10242,6 @@
           <t>Sky Blue Jacquard Full Sleeves Rich Floral Embroidery Sherwani</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122635/zoddle/img-89eb9dc4.jpg</t>
@@ -10377,13 +10257,11 @@
           <t>https://www.myntra.com/sherwani/aj+dezines/aj-dezines-boys-embroidered-sherwani-set-/37905885/buy</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0GJ5ZW7TQ</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -10417,7 +10295,6 @@
           <t>Boys Purple Cotton Full Sleeves Floral Print Kurta Pyjama Set</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122641/zoddle/img-491ff08a.jpg</t>
@@ -10433,8 +10310,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-floral-printed-long-sleeves-pure-cotton-straight-kurta-with-trouser/36003124/buy</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-boys-festive-party-kurta-pyjama-set/p/itm05168be423ac3</t>
@@ -10473,16 +10348,11 @@
           <t>Black Full Sleeves Floral Print Cotton Kurta Pyjama (1272)</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122638/zoddle/img-44cf3a04.jpg</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/aj-dezines-baby-boys-festive-party-kurta-pyjama-set/p/itm6b87a3bc004dd</t>
@@ -10521,7 +10391,6 @@
           <t>Kids Boys Blue Floral Print Cotton Suit Set (3-piece KPW)</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1780122654/zoddle/img-5df9b012.jpg</t>
@@ -10537,7 +10406,6 @@
           <t>https://www.myntra.com/kurta-sets/aj+dezines/aj-dezines-boys-floral-printed-zari-pure-cotton-kurta-with-pyjamas--nehru-jacket/22218402/buy</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CHP2CN26</t>
@@ -10769,4 +10637,3211 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>zoddle_barcode</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>design_code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>brand_size</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>zoddle_price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>mrp</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>design_name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>colour</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Myntra</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>FirstCry</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Flipkart</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>last_updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>27460134</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2746</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>1445</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Orange &amp; Pink Embroidered Choli &amp; Ready to Wear Lehenga With Dupatta</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-aa1256c5.webp</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-orange-pink-embroidered-choli-ready-to-wear-lehenga-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-foil-print-ready-to-wear-lehenga--blouse-with-dupatta/33629580/buy</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6HBS78</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>27460156</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2746</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>1445</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Orange &amp; Pink Embroidered Choli &amp; Ready to Wear Lehenga With Dupatta</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-aa1256c5.webp</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-orange-pink-embroidered-choli-ready-to-wear-lehenga-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-foil-print-ready-to-wear-lehenga--blouse-with-dupatta/33629580/buy</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6HBS78</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>27460178</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2746</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>1445</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Orange &amp; Pink Embroidered Choli &amp; Ready to Wear Lehenga With Dupatta</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-aa1256c5.webp</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-orange-pink-embroidered-choli-ready-to-wear-lehenga-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-foil-print-ready-to-wear-lehenga--blouse-with-dupatta/33629580/buy</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6HBS78</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>27470134</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2747</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>1359</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Jacquard booti Lehenga Choli Ready to Wear with Pink Dupatta</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599396/zoddle/img-32d7672f.jpg</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-jacquard-booti-lehenga-choli-ready-to-wear-with-pink-dupatta-tlhc107</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-ready-to-wear-lehenga--blouse-with-dupatta/25156664/buy</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J65MV</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>27470156</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2747</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>1359</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Jacquard booti Lehenga Choli Ready to Wear with Pink Dupatta</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599396/zoddle/img-32d7672f.jpg</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-jacquard-booti-lehenga-choli-ready-to-wear-with-pink-dupatta-tlhc107</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-ready-to-wear-lehenga--blouse-with-dupatta/25156664/buy</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J65MV</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>27470178</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2747</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>1359</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Jacquard booti Lehenga Choli Ready to Wear with Pink Dupatta</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599396/zoddle/img-32d7672f.jpg</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-jacquard-booti-lehenga-choli-ready-to-wear-with-pink-dupatta-tlhc107</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-ready-to-wear-lehenga--blouse-with-dupatta/25156664/buy</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J65MV</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>27480134</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2748</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>1530</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Floral Print Top &amp; Shrug With Ready to wear Skirts</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599415/zoddle/img-8ff9d225.webp</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-floral-print-top-shrug-with-ready-to-wear-skirts-tlhc098</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-ready-to-wear-lehenga--blouse-with-shrug/24817552/buy</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-floral-printed-gota-lace-embellished-lehenga-choli-with-three-fourth-sleeves-shrug-set-yellow/20717746/product-detail</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J2Z3M</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmbb6e72da0f747</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>27480156</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2748</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>1530</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Floral Print Top &amp; Shrug With Ready to wear Skirts</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599415/zoddle/img-8ff9d225.webp</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-floral-print-top-shrug-with-ready-to-wear-skirts-tlhc098</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-ready-to-wear-lehenga--blouse-with-shrug/24817552/buy</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-floral-printed-gota-lace-embellished-lehenga-choli-with-three-fourth-sleeves-shrug-set-yellow/20717746/product-detail</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J2Z3M</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmbb6e72da0f747</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>27490134</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2749</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>1662</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Pink embroidered Choli &amp; Pink Jaquard booti Design Lehenga With Dupatta</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599417/zoddle/img-4b217b24.webp</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-pink-embroidered-choli-pink-jaquard-booti-design-lehenga-with-dupatta-tlhc129</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-ready-to-wear-lehenga--blouse-with-dupatta/25189506/buy</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-sleeveless-sequins-embellished-and-floral-embroidered-flared-lehenga-choli-set-with-dupatta-pink/23909972/product-detail</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J37HN</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmec3f7ef8003af</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>27490156</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2749</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>1662</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Pink embroidered Choli &amp; Pink Jaquard booti Design Lehenga With Dupatta</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599417/zoddle/img-4b217b24.webp</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-pink-embroidered-choli-pink-jaquard-booti-design-lehenga-with-dupatta-tlhc129</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-ready-to-wear-lehenga--blouse-with-dupatta/25189506/buy</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-sleeveless-sequins-embellished-and-floral-embroidered-flared-lehenga-choli-set-with-dupatta-pink/23909972/product-detail</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J37HN</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmec3f7ef8003af</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>27490178</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2749</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>1662</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Pink embroidered Choli &amp; Pink Jaquard booti Design Lehenga With Dupatta</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599417/zoddle/img-4b217b24.webp</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-pink-embroidered-choli-pink-jaquard-booti-design-lehenga-with-dupatta-tlhc129</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-ready-to-wear-lehenga--blouse-with-dupatta/25189506/buy</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-sleeveless-sequins-embellished-and-floral-embroidered-flared-lehenga-choli-set-with-dupatta-pink/23909972/product-detail</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J37HN</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmec3f7ef8003af</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>27500134</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2750</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>999</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Green &amp; Pink Woven Design Choli - Ready to Wear Lehenga with Dupatta</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-54030ec4.webp</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-green-pink-woven-design-choli-ready-to-wear-lehenga-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-ready-to-wear-lehenga--blouse-with-dupatta/33809828/buy</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J53VT</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>27500156</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2750</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="n">
+        <v>999</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Green &amp; Pink Woven Design Choli - Ready to Wear Lehenga with Dupatta</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-54030ec4.webp</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-green-pink-woven-design-choli-ready-to-wear-lehenga-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-ready-to-wear-lehenga--blouse-with-dupatta/33809828/buy</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J53VT</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>27500178</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2750</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Green &amp; Pink Woven Design Choli - Ready to Wear Lehenga with Dupatta</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-54030ec4.webp</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-green-pink-woven-design-choli-ready-to-wear-lehenga-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-ready-to-wear-lehenga--blouse-with-dupatta/33809828/buy</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6J53VT</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>27510134</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2751</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>1690</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow with Embroidered Ready to Wear Lehenga &amp; Choli with Dupatta.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-6d6f0f5e.webp</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-with-embroidered-ready-to-wear-lehenga-choli-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-floral-embroidered-ready-to-wear-lehenga--blouse-with-dupatta/36955604/buy</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21214523/product-detail</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTVBMKQ3</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-indi-girls-lehenga-choli-ethnic-wear-embroidered/p/itmf12911d6dcec5</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>27510156</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2751</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>1690</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow with Embroidered Ready to Wear Lehenga &amp; Choli with Dupatta.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-6d6f0f5e.webp</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-with-embroidered-ready-to-wear-lehenga-choli-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-floral-embroidered-ready-to-wear-lehenga--blouse-with-dupatta/36955604/buy</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21214523/product-detail</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTVBMKQ3</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-indi-girls-lehenga-choli-ethnic-wear-embroidered/p/itmf12911d6dcec5</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>27510178</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2751</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>1690</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow with Embroidered Ready to Wear Lehenga &amp; Choli with Dupatta.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-6d6f0f5e.webp</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-with-embroidered-ready-to-wear-lehenga-choli-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-floral-embroidered-ready-to-wear-lehenga--blouse-with-dupatta/36955604/buy</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21214523/product-detail</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTVBMKQ3</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-indi-girls-lehenga-choli-ethnic-wear-embroidered/p/itmf12911d6dcec5</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>27520134</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2752</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Ready to wear Choli &amp; Lehenga</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-0692492f.webp</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-ready-to-wear-choli-lehenga</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6CK43T</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmb11959e5e5895</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>27520156</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2752</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Ready to wear Choli &amp; Lehenga</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-0692492f.webp</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-ready-to-wear-choli-lehenga</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6CK43T</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmb11959e5e5895</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>27520178</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2752</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Ready to wear Choli &amp; Lehenga</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599412/zoddle/img-0692492f.webp</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-ready-to-wear-choli-lehenga</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6CK43T</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-lehenga-choli-ethnic-wear-printed/p/itmb11959e5e5895</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>27530134</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2753</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>1611</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4999</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Orange &amp; Pink with Embroidered Ready to Wear Lehenga &amp; Choli with Dupatta.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-910c048e.webp</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-orange-pink-with-embroidered-ready-to-wear-lehenga-choli-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-zari-ready-to-wear-lehenga--blouse-with-dupatta/36955614/buy</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/23910087/product-detail</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTVDGQS8</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>27530156</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2753</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>1611</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4999</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Orange &amp; Pink with Embroidered Ready to Wear Lehenga &amp; Choli with Dupatta.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-910c048e.webp</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-orange-pink-with-embroidered-ready-to-wear-lehenga-choli-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-zari-ready-to-wear-lehenga--blouse-with-dupatta/36955614/buy</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/23910087/product-detail</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTVDGQS8</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>27530178</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2753</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>1611</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4999</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Orange &amp; Pink with Embroidered Ready to Wear Lehenga &amp; Choli with Dupatta.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-910c048e.webp</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-orange-pink-with-embroidered-ready-to-wear-lehenga-choli-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-zari-ready-to-wear-lehenga--blouse-with-dupatta/36955614/buy</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/23910087/product-detail</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTVDGQS8</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>27540134</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2754</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>1530</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Bitiya By Bhama Girls Pink Flower Digital Multi Print Lace Work Choli With Ready To Wear Lehenga.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599414/zoddle/img-b04b731a.webp</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-pink-flower-digital-multi-print-lace-work-choli-with-ready-to-wear-lehenga-tlhc093</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-printed-ready-to-wear-lehenga/22752698/buy</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6H2GW3</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>27540156</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2754</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>1530</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Bitiya By Bhama Girls Pink Flower Digital Multi Print Lace Work Choli With Ready To Wear Lehenga.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599414/zoddle/img-b04b731a.webp</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-pink-flower-digital-multi-print-lace-work-choli-with-ready-to-wear-lehenga-tlhc093</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-printed-ready-to-wear-lehenga/22752698/buy</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6H2GW3</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>27540178</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2754</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>1530</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Bitiya By Bhama Girls Pink Flower Digital Multi Print Lace Work Choli With Ready To Wear Lehenga.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599414/zoddle/img-b04b731a.webp</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-pink-flower-digital-multi-print-lace-work-choli-with-ready-to-wear-lehenga-tlhc093</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/lehenga-choli/bitiya+by+bhama/bitiya-by-bhama-girls-printed-ready-to-wear-lehenga/22752698/buy</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FH6H2GW3</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27550134</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2755</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>1641</v>
+      </c>
+      <c r="F28" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Multi Floral Angrakha Gotta Patti Kurta Sharara set With Dupatta</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-efb9cddf.webp</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-multi-floral-angrakha-gotta-patti-kurta-sharara-set-with-dupatta-tks136</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-angrakha-anarkali-kurta--sharara-with-dupatta/24188486/buy</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQK31X6</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-pyjama-dupatta-set/p/itm951c99eb38dc3</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>27550156</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2755</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>1641</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Multi Floral Angrakha Gotta Patti Kurta Sharara set With Dupatta</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-efb9cddf.webp</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-multi-floral-angrakha-gotta-patti-kurta-sharara-set-with-dupatta-tks136</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-angrakha-anarkali-kurta--sharara-with-dupatta/24188486/buy</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQK31X6</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-pyjama-dupatta-set/p/itm951c99eb38dc3</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>27550178</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2755</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>1641</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Yellow Multi Floral Angrakha Gotta Patti Kurta Sharara set With Dupatta</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-efb9cddf.webp</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-yellow-multi-floral-angrakha-gotta-patti-kurta-sharara-set-with-dupatta-tks136</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-angrakha-anarkali-kurta--sharara-with-dupatta/24188486/buy</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQK31X6</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-pyjama-dupatta-set/p/itm951c99eb38dc3</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>27560134</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2756</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Bitiya By Bhama Girls Pink Embroidered Kurta With Trousers &amp; With Dupatta</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-da014eb5.webp</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-blue-embroidered-kurta-with-trousers-with-dupatta-tks075</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-angrakha-kurta-with-trousers--dupatta/21570842/buy</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-three-fourth-sleeves-floral-embroidered-kurta-and-pant-with-dupatta-set-pink/20733542/product-detail</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQGT1JK</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-pyjama-dupatta-set/p/itmaccba4e5ec0e0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>27560156</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2756</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Bitiya By Bhama Girls Pink Embroidered Kurta With Trousers &amp; With Dupatta</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-da014eb5.webp</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-blue-embroidered-kurta-with-trousers-with-dupatta-tks075</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-angrakha-kurta-with-trousers--dupatta/21570842/buy</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-three-fourth-sleeves-floral-embroidered-kurta-and-pant-with-dupatta-set-pink/20733542/product-detail</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQGT1JK</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-pyjama-dupatta-set/p/itmaccba4e5ec0e0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>27560178</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2756</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F33" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Bitiya By Bhama Girls Pink Embroidered Kurta With Trousers &amp; With Dupatta</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599413/zoddle/img-da014eb5.webp</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-blue-embroidered-kurta-with-trousers-with-dupatta-tks075</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-angrakha-kurta-with-trousers--dupatta/21570842/buy</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-three-fourth-sleeves-floral-embroidered-kurta-and-pant-with-dupatta-set-pink/20733542/product-detail</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQGT1JK</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-pyjama-dupatta-set/p/itmaccba4e5ec0e0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>27570134</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2757</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>1299</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Embroidered Angrakha Kurta with Trousers &amp; Dupatta</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599414/zoddle/img-fd05fee7.webp</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-embroidered-angrakha-kurta-with-trousers-dupatta-tks111</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-angrakha-gotta-patti-kurta-with-trousers--dupatta/23447862/buy</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-three-fourth-sleeves-floral-embroidered-anarkali-kurti-and-palazzo-with-dupatta-set-peach/20555201/product-detail</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQB5B3Z</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-palazzo-set/p/itm307192458aaca</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>27570156</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2757</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>1299</v>
+      </c>
+      <c r="F35" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Embroidered Angrakha Kurta with Trousers &amp; Dupatta</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599414/zoddle/img-fd05fee7.webp</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-embroidered-angrakha-kurta-with-trousers-dupatta-tks111</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-angrakha-gotta-patti-kurta-with-trousers--dupatta/23447862/buy</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-three-fourth-sleeves-floral-embroidered-anarkali-kurti-and-palazzo-with-dupatta-set-peach/20555201/product-detail</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQB5B3Z</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-palazzo-set/p/itm307192458aaca</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>27570178</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2757</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>1299</v>
+      </c>
+      <c r="F36" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Embroidered Angrakha Kurta with Trousers &amp; Dupatta</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599414/zoddle/img-fd05fee7.webp</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-embroidered-angrakha-kurta-with-trousers-dupatta-tks111</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-embroidered-angrakha-gotta-patti-kurta-with-trousers--dupatta/23447862/buy</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bitiya-by-bhama/bitiya-by-bhama-silk-woven-three-fourth-sleeves-floral-embroidered-anarkali-kurti-and-palazzo-with-dupatta-set-peach/20555201/product-detail</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FHQB5B3Z</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-palazzo-set/p/itm307192458aaca</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>27580134</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2758</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>1550</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Ethnic motifs woven design Kurta With Sharara &amp; With Dupatta</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599411/zoddle/img-a7cede2b.webp</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-ethnic-motifs-woven-design-kurta-with-sharara-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-ethnic-motifs-woven-design-sequinned-kurta-with-sharara--dupatta/36977814/buy</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTS7P4KX</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-sharara-set/p/itme87ef93bf70a1</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>27580156</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2758</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>1550</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Ethnic motifs woven design Kurta With Sharara &amp; With Dupatta</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599411/zoddle/img-a7cede2b.webp</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-ethnic-motifs-woven-design-kurta-with-sharara-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-ethnic-motifs-woven-design-sequinned-kurta-with-sharara--dupatta/36977814/buy</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTS7P4KX</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-sharara-set/p/itme87ef93bf70a1</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>27580178</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2758</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>1550</v>
+      </c>
+      <c r="F39" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls Ethnic motifs woven design Kurta With Sharara &amp; With Dupatta</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599411/zoddle/img-a7cede2b.webp</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-ethnic-motifs-woven-design-kurta-with-sharara-with-dupatta</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-ethnic-motifs-woven-design-sequinned-kurta-with-sharara--dupatta/36977814/buy</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTS7P4KX</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-sharara-set/p/itme87ef93bf70a1</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>27590134</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2759</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>699</v>
+      </c>
+      <c r="F40" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls purple Angrakha Gotta Patti Kurta with Sharara</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599411/zoddle/img-a6298bb6.webp</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-purple-angrakha-gotta-patti-kurta-with-sharara</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-angrakha-anarkali-pure-cotton-kurta-with-sharara/36977837/buy</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTS7NR58</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-sharara-set/p/itm0795816288da1</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>27590156</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2759</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>699</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls purple Angrakha Gotta Patti Kurta with Sharara</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599411/zoddle/img-a6298bb6.webp</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-purple-angrakha-gotta-patti-kurta-with-sharara</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-angrakha-anarkali-pure-cotton-kurta-with-sharara/36977837/buy</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTS7NR58</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-sharara-set/p/itm0795816288da1</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>27590178</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2759</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>699</v>
+      </c>
+      <c r="F42" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Bitiya by Bhama Girls purple Angrakha Gotta Patti Kurta with Sharara</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599411/zoddle/img-a6298bb6.webp</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bitiya-by-bhama-girls-purple-angrakha-gotta-patti-kurta-with-sharara</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bitiya+by+bhama/bitiya-by-bhama-girls-floral-printed-angrakha-anarkali-pure-cotton-kurta-with-sharara/36977837/buy</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0FTS7NR58</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bitiya-bhama-girls-festive-party-kurta-sharara-set/p/itm0795816288da1</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>27600134</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2760</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>1140</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Bittu By Bhama Boys off white kurta pajama with a jacquard booti jacket</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599410/zoddle/img-a009b392.webp</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bittu-by-bhama-boys-off-white-kurta-pajama-with-a-jacquard-booti-jacket</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bittu+by+bhama/bittu-by-bhama-boys-floral-printed-kurta-with-pyjama--nehru-jacket/37003898/buy</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/bittu-by-bhama/bittu-by-bhama-cotton-blend-woven-full-sleeves-solid-kurta-pyjama-with-floral-printed-jacket-set-off-white/21306571/product-detail</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bittu-bhama-boys-festive-party-kurta-pyjama-set/p/itm971cbc5c299be</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>27610134</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2761</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>3-4Y</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>1188</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Bittu By Bhama Boys Pink floral printed kurta with a Pink pajama.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599410/zoddle/img-6bbc4a4b.webp</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bittu-by-bhama-boys-pink-floral-printed-kurta-with-a-pink-pajama</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bittu+by+bhama/bittu-by-bhama-boys-floral-printed-mandarin-collar-regular-kurta-with-pyjamas/37003932/buy</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21306544/product-detail</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bittu-bhama-boys-festive-party-kurta-pyjama-set/p/itmac0834dbce31c</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>27610156</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2761</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>1188</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Bittu By Bhama Boys Pink floral printed kurta with a Pink pajama.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599410/zoddle/img-6bbc4a4b.webp</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bittu-by-bhama-boys-pink-floral-printed-kurta-with-a-pink-pajama</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bittu+by+bhama/bittu-by-bhama-boys-floral-printed-mandarin-collar-regular-kurta-with-pyjamas/37003932/buy</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21306544/product-detail</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bittu-bhama-boys-festive-party-kurta-pyjama-set/p/itmac0834dbce31c</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>27610178</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2761</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="n">
+        <v>1188</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Bittu By Bhama Boys Pink floral printed kurta with a Pink pajama.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599410/zoddle/img-6bbc4a4b.webp</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bittu-by-bhama-boys-pink-floral-printed-kurta-with-a-pink-pajama</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bittu+by+bhama/bittu-by-bhama-boys-floral-printed-mandarin-collar-regular-kurta-with-pyjamas/37003932/buy</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21306544/product-detail</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bittu-bhama-boys-festive-party-kurta-pyjama-set/p/itmac0834dbce31c</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>27620156</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2762</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>5-6Y</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>1155</v>
+      </c>
+      <c r="F47" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Bittu By Bhama Boys yellow &amp; red kurta with a white pajama</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599410/zoddle/img-b7701f82.webp</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bittu-by-bhama-boys-yellow-red-kurta-with-a-white-pajama</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bittu+by+bhama/bittu-by-bhama-boys-ethnic-motifs-floral-printed-regular-kurta-with-pyjamas/37003916/buy</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21306621/product-detail</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bittu-bhama-boys-festive-party-kurta-pyjama-set/p/itm3213c6b5a0665</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>27620178</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2762</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7-8Y</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>1155</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Bittu By Bhama Boys yellow &amp; red kurta with a white pajama</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dxy6fdqsa/image/upload/v1790599410/zoddle/img-b7701f82.webp</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://www.bhamadesigns.com/products/bittu-by-bhama-boys-yellow-red-kurta-with-a-white-pajama</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>https://www.myntra.com/kurta-sets/bittu+by+bhama/bittu-by-bhama-boys-ethnic-motifs-floral-printed-regular-kurta-with-pyjamas/37003916/buy</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.firstcry.com/x/x/21306621/product-detail</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/bittu-bhama-boys-festive-party-kurta-pyjama-set/p/itm3213c6b5a0665</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId234"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>